<commit_message>
Implented v, T, and P data storage for MotorPropAssy.m
- Also worked on analyzing stall, cruise, and max speeds for different angles of attack
- Chopped off angles of attack in airfoil c_l spreadsheet past linear region (cl no longer linear w alpha)
</commit_message>
<xml_diff>
--- a/Propulsion & Power/Tabulated Airfoil c_l Values/E210_c_l.xlsx
+++ b/Propulsion & Power/Tabulated Airfoil c_l Values/E210_c_l.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mailmissouri-my.sharepoint.com/personal/arvkb9_umsystem_edu/Documents/896 - B.S Aerospace Engineering Courses/92 - Fall 2026/6 - AE4780-Meeks/Github Repo/Miner-Works-MW-27-MantaRay/Propulsion &amp; Power/Tabulated Airfoil c_l Values/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{DC56BE96-02B0-466A-A13D-84E50E3BCDC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40A607AE-634C-439F-8A6A-6DE4F4D49F37}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="8_{DC56BE96-02B0-466A-A13D-84E50E3BCDC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{363FE127-6D5F-45FF-9617-5CD1C7656CC4}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{706E62A6-5DB7-4E23-AC7D-EF51E1E871E8}"/>
   </bookViews>
@@ -569,6 +569,2159 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>NACA2412_c_l!$A$2:$A$71</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="70"/>
+                <c:pt idx="0">
+                  <c:v>-10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-9.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-9</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-8.5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-8</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-7.5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-6.5</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-6</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-5.5</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-5</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>-4.5</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>-3.5</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>-3</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>-2.5</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-1.5</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-1</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-0.5</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>1.5</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>2.5</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>3.5</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>4.5</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>5.5</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>6.5</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>7.5</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>8.5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>NACA2412_c_l!$B$2:$B$71</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="70"/>
+                <c:pt idx="0">
+                  <c:v>-0.36930000000000002</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-0.40200000000000002</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-0.4768</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.4577</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.39600000000000002</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-0.32769999999999999</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-0.28370000000000001</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-0.21249999999999999</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-0.1605</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-7.7399999999999997E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-5.8999999999999999E-3</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>6.2899999999999998E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.1724</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.22409999999999999</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.27910000000000001</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.33300000000000002</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.3866</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.44030000000000002</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.49399999999999999</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.54920000000000002</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.60419999999999996</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.65780000000000005</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.71309999999999996</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.76590000000000003</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.81850000000000001</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.91720000000000002</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.9728</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>1.0266</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>1.0787</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>1.1288</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>1.1706000000000001</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>1.2128000000000001</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>1.2572000000000001</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>1.2927999999999999</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>1.3190999999999999</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>1.3562000000000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-FE33-4A33-BDB5-1335BC328A04}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1506466224"/>
+        <c:axId val="1898175408"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1506466224"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1898175408"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1898175408"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1506466224"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>NACA2412_c_l!$A$12:$A$40</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="29"/>
+                <c:pt idx="0">
+                  <c:v>-5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-4.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-3.5</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-2.5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-1.5</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-1</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-0.5</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.5</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.5</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>3.5</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>4.5</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>5.5</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>6.5</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>7.5</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>8.5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>NACA2412_c_l!$B$12:$B$40</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="29"/>
+                <c:pt idx="0">
+                  <c:v>-5.8999999999999999E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6.2899999999999998E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.1724</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.22409999999999999</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.27910000000000001</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.33300000000000002</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.3866</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.44030000000000002</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.49399999999999999</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.54920000000000002</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.60419999999999996</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.65780000000000005</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.71309999999999996</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.76590000000000003</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.81850000000000001</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.91720000000000002</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.9728</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1.0266</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1.0787</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1.1288</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1.1706000000000001</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>1.2128000000000001</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>1.2572000000000001</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>1.2927999999999999</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>1.3190999999999999</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>1.3562000000000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-9AE5-4F67-83F5-2196E29B62A5}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="427146688"/>
+        <c:axId val="1898119728"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="427146688"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1898119728"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1898119728"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="427146688"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>236220</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>541020</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7EA265A7-57ED-AABB-0BDF-37AFBB733592}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>297543</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>140245</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>609600</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>140245</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{57D4FC45-A7E7-8551-9F69-F9B5F098077F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -886,7 +3039,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{784AA86F-C3BA-47F6-A64C-FE3BBE194E9E}">
-  <dimension ref="A1:B71"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -1185,279 +3338,8 @@
         <v>1.3562000000000001</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A38">
-        <v>9</v>
-      </c>
-      <c r="B38">
-        <v>1.3732</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A39">
-        <v>9.5</v>
-      </c>
-      <c r="B39">
-        <v>1.3874</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A40">
-        <v>10</v>
-      </c>
-      <c r="B40">
-        <v>1.4000999999999999</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A41">
-        <v>10.5</v>
-      </c>
-      <c r="B41">
-        <v>1.4047000000000001</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A42">
-        <v>11</v>
-      </c>
-      <c r="B42">
-        <v>1.3917999999999999</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A43">
-        <v>11.5</v>
-      </c>
-      <c r="B43">
-        <v>1.4009</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A44">
-        <v>12</v>
-      </c>
-      <c r="B44">
-        <v>1.4087000000000001</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A45">
-        <v>12.5</v>
-      </c>
-      <c r="B45">
-        <v>1.4135</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A46">
-        <v>13</v>
-      </c>
-      <c r="B46">
-        <v>1.413</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A47">
-        <v>13.5</v>
-      </c>
-      <c r="B47">
-        <v>1.407</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A48">
-        <v>14</v>
-      </c>
-      <c r="B48">
-        <v>1.3936999999999999</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A49">
-        <v>14.5</v>
-      </c>
-      <c r="B49">
-        <v>1.3806</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50">
-        <v>15</v>
-      </c>
-      <c r="B50">
-        <v>1.3655999999999999</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A51">
-        <v>15.5</v>
-      </c>
-      <c r="B51">
-        <v>1.351</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A52">
-        <v>16</v>
-      </c>
-      <c r="B52">
-        <v>1.3411</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A53">
-        <v>16.5</v>
-      </c>
-      <c r="B53">
-        <v>1.3304</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A54">
-        <v>17</v>
-      </c>
-      <c r="B54">
-        <v>1.3185</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A55">
-        <v>17.5</v>
-      </c>
-      <c r="B55">
-        <v>1.3026</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A56">
-        <v>18</v>
-      </c>
-      <c r="B56">
-        <v>1.2786</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A57">
-        <v>18.5</v>
-      </c>
-      <c r="B57">
-        <v>1.2495000000000001</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A58">
-        <v>19</v>
-      </c>
-      <c r="B58">
-        <v>1.2169000000000001</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A59">
-        <v>19.5</v>
-      </c>
-      <c r="B59">
-        <v>1.1805000000000001</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A60">
-        <v>20</v>
-      </c>
-      <c r="B60">
-        <v>1.1373</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A61">
-        <v>20.5</v>
-      </c>
-      <c r="B61">
-        <v>1.0644</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A62">
-        <v>21</v>
-      </c>
-      <c r="B62">
-        <v>1.0135000000000001</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A63">
-        <v>21.5</v>
-      </c>
-      <c r="B63">
-        <v>0.93500000000000005</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A64">
-        <v>22</v>
-      </c>
-      <c r="B64">
-        <v>0.91049999999999998</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A65">
-        <v>22.5</v>
-      </c>
-      <c r="B65">
-        <v>0.89600000000000002</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A66">
-        <v>23</v>
-      </c>
-      <c r="B66">
-        <v>0.88690000000000002</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A67">
-        <v>23.5</v>
-      </c>
-      <c r="B67">
-        <v>0.88239999999999996</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A68">
-        <v>24</v>
-      </c>
-      <c r="B68">
-        <v>0.87649999999999995</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A69">
-        <v>24.5</v>
-      </c>
-      <c r="B69">
-        <v>0.87180000000000002</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A70">
-        <v>25</v>
-      </c>
-      <c r="B70">
-        <v>0.86809999999999998</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A71">
-        <v>25.5</v>
-      </c>
-      <c r="B71">
-        <v>0.86550000000000005</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>